<commit_message>
chore: regenerate Achmea_2025_Databook.xlsx with corrected extraction
Rebuilt using fixed page maps and prompts: Note 7 movement tables now
use 2025-only pages, CSM prompt matches embedded GMM column structure,
and discount rate extraction targets the correct pages (276-277) with
Dutch decimal and min-max range handling.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Achmea_2025_Databook.xlsx
+++ b/Achmea_2025_Databook.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="212">
   <si>
     <t xml:space="preserve">Mapping Financial Statements - Achmea Dataset</t>
   </si>
@@ -221,22 +221,25 @@
     <t xml:space="preserve">c) Supplementary information</t>
   </si>
   <si>
-    <t xml:space="preserve">i) Last Liquid point (years)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ii) Long Term Forward Rate</t>
+    <t xml:space="preserve">ii) Ultimate Forward Rate (UFR)</t>
   </si>
   <si>
     <t xml:space="preserve">Cost of capital rate</t>
   </si>
   <si>
-    <t xml:space="preserve">Confidence level - Life</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confidence level - Non-Life</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confidence level - Health</t>
+    <t xml:space="preserve">Pg.276</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confidence level - Life NL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pg.277</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confidence level - Non-Life NL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confidence level - Health NL</t>
   </si>
   <si>
     <t xml:space="preserve">(3) LRC AND LIC DEEP-DIVE</t>
@@ -254,100 +257,91 @@
     <t xml:space="preserve">b.1) New business</t>
   </si>
   <si>
+    <t xml:space="preserve">c) Insurance finance results</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d) Future service changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e) CSM release</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g) Other</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h) Closing balance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSM DEVELOPMENT WITH SPLIT:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A) Opening balance (Non-Life GMM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note 7 [Pg.259]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B) Opening balance (Life GMM &amp; VFA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note 7 [Pg.269-270]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  [Health GMM not separately disclosed — PAA-dominated portfolio]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A.1) New business (Non-Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B.1) New business (Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A.3) Finance (Non-Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B.3) Finance (Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A.4) Future service (Non-Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B.4) Future service (Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A.6) CSM release (Non-Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B.6) CSM release (Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A.8) Other (Non-Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B.8) Other (Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A) Closing balance (Non-Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B) Closing balance (Life)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(i.b) CSM RELEASE MATURITY:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a) 0-1 year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note 7 [Pg.254]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b) 1-5 years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(ii.a) OVERVIEW OF RISK ADJUSTMENT DEVELOPMENT:</t>
+  </si>
+  <si>
     <t xml:space="preserve">b.2) Acquisitions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c) Insurance finance results</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d) Future service changes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">e) CSM release</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f) Foreign currency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">g) Other</t>
-  </si>
-  <si>
-    <t xml:space="preserve">h) Closing balance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CSM DEVELOPMENT WITH SPLIT:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A) Opening balance (Non-Life GMM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note 7 [Pg.259-260]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B) Opening balance (Life GMM &amp; VFA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note 7 [Pg.269-270]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C) Opening balance (Health)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A.1) New business (Non-Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B.1) New business (Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A.3) Finance (Non-Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B.3) Finance (Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A.4) Future service (Non-Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B.4) Future service (Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A.6) CSM release (Non-Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B.6) CSM release (Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C.6) CSM release (Health)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A.8) Other (Non-Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B.8) Other (Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A) Closing balance (Non-Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B) Closing balance (Life)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C) Closing balance (Health)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(i.b) CSM RELEASE MATURITY:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a) 0-1 year</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note 7 [Pg.254]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b) 1-5 years</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(ii.a) OVERVIEW OF RISK ADJUSTMENT DEVELOPMENT:</t>
   </si>
   <si>
     <t xml:space="preserve">c) Insurance finance</t>
@@ -1575,6 +1569,9 @@
       <c r="A67" t="s">
         <v>58</v>
       </c>
+      <c r="B67" t="n">
+        <v>0.0229</v>
+      </c>
       <c r="C67"/>
       <c r="D67"/>
       <c r="E67" t="s">
@@ -1585,6 +1582,9 @@
       <c r="A68" t="s">
         <v>60</v>
       </c>
+      <c r="B68" t="n">
+        <v>0.0275</v>
+      </c>
       <c r="C68"/>
       <c r="D68"/>
       <c r="E68" t="s">
@@ -1595,6 +1595,9 @@
       <c r="A69" t="s">
         <v>61</v>
       </c>
+      <c r="B69" t="n">
+        <v>0.03145</v>
+      </c>
       <c r="C69"/>
       <c r="D69"/>
       <c r="E69" t="s">
@@ -1605,6 +1608,9 @@
       <c r="A70" t="s">
         <v>62</v>
       </c>
+      <c r="B70" t="n">
+        <v>0.03395</v>
+      </c>
       <c r="C70"/>
       <c r="D70"/>
       <c r="E70" t="s">
@@ -1615,6 +1621,9 @@
       <c r="A71" t="s">
         <v>63</v>
       </c>
+      <c r="B71" t="n">
+        <v>0.03505</v>
+      </c>
       <c r="C71"/>
       <c r="D71"/>
       <c r="E71" t="s">
@@ -1625,6 +1634,9 @@
       <c r="A72" t="s">
         <v>64</v>
       </c>
+      <c r="B72" t="n">
+        <v>0.03495</v>
+      </c>
       <c r="C72"/>
       <c r="D72"/>
       <c r="E72" t="s">
@@ -1635,6 +1647,9 @@
       <c r="A73" t="s">
         <v>65</v>
       </c>
+      <c r="B73" t="n">
+        <v>0.03185</v>
+      </c>
       <c r="C73"/>
       <c r="D73"/>
       <c r="E73" t="s">
@@ -1650,6 +1665,9 @@
       <c r="A76" t="s">
         <v>58</v>
       </c>
+      <c r="B76" t="n">
+        <v>0.0233</v>
+      </c>
       <c r="C76"/>
       <c r="D76"/>
       <c r="E76" t="s">
@@ -1660,6 +1678,9 @@
       <c r="A77" t="s">
         <v>60</v>
       </c>
+      <c r="B77" t="n">
+        <v>0.0274</v>
+      </c>
       <c r="C77"/>
       <c r="D77"/>
       <c r="E77" t="s">
@@ -1670,6 +1691,9 @@
       <c r="A78" t="s">
         <v>61</v>
       </c>
+      <c r="B78" t="n">
+        <v>0.03135</v>
+      </c>
       <c r="C78"/>
       <c r="D78"/>
       <c r="E78" t="s">
@@ -1680,6 +1704,9 @@
       <c r="A79" t="s">
         <v>62</v>
       </c>
+      <c r="B79" t="n">
+        <v>0.0339</v>
+      </c>
       <c r="C79"/>
       <c r="D79"/>
       <c r="E79" t="s">
@@ -1690,6 +1717,9 @@
       <c r="A80" t="s">
         <v>63</v>
       </c>
+      <c r="B80" t="n">
+        <v>0.0347</v>
+      </c>
       <c r="C80"/>
       <c r="D80"/>
       <c r="E80" t="s">
@@ -1700,6 +1730,9 @@
       <c r="A81" t="s">
         <v>64</v>
       </c>
+      <c r="B81" t="n">
+        <v>0.03445</v>
+      </c>
       <c r="C81"/>
       <c r="D81"/>
       <c r="E81" t="s">
@@ -1710,6 +1743,9 @@
       <c r="A82" t="s">
         <v>65</v>
       </c>
+      <c r="B82" t="n">
+        <v>0.0312</v>
+      </c>
       <c r="C82"/>
       <c r="D82"/>
       <c r="E82" t="s">
@@ -1725,540 +1761,595 @@
       <c r="A85" t="s">
         <v>69</v>
       </c>
+      <c r="B85" t="n">
+        <v>0.023</v>
+      </c>
       <c r="C85"/>
       <c r="D85"/>
       <c r="E85" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
         <v>70</v>
       </c>
+      <c r="B86" t="n">
+        <v>0.045</v>
+      </c>
       <c r="C86"/>
       <c r="D86"/>
       <c r="E86" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>71</v>
+        <v>72</v>
+      </c>
+      <c r="B87" t="n">
+        <v>0.861</v>
       </c>
       <c r="C87"/>
       <c r="D87"/>
       <c r="E87" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>72</v>
+        <v>74</v>
+      </c>
+      <c r="B88" t="n">
+        <v>0.721</v>
       </c>
       <c r="C88"/>
       <c r="D88"/>
       <c r="E88" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>73</v>
+        <v>75</v>
+      </c>
+      <c r="B89" t="n">
+        <v>0.551</v>
       </c>
       <c r="C89"/>
       <c r="D89"/>
       <c r="E89" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="s">
-        <v>74</v>
-      </c>
-      <c r="C90"/>
-      <c r="D90"/>
-      <c r="E90" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="s">
-        <v>76</v>
+      <c r="A95" t="s">
+        <v>78</v>
+      </c>
+      <c r="B95" t="n">
+        <v>1140</v>
+      </c>
+      <c r="C95"/>
+      <c r="D95"/>
+      <c r="E95" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>77</v>
+        <v>80</v>
+      </c>
+      <c r="B96" t="n">
+        <v>15</v>
       </c>
       <c r="C96"/>
       <c r="D96"/>
       <c r="E96" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>79</v>
+        <v>81</v>
+      </c>
+      <c r="B97" t="n">
+        <v>34</v>
       </c>
       <c r="C97"/>
       <c r="D97"/>
       <c r="E97" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B98" t="n">
-        <v>55</v>
+        <v>-160</v>
       </c>
       <c r="C98"/>
       <c r="D98"/>
       <c r="E98" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>81</v>
+        <v>83</v>
+      </c>
+      <c r="B99" t="n">
+        <v>-76</v>
       </c>
       <c r="C99"/>
       <c r="D99"/>
       <c r="E99" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>82</v>
+        <v>84</v>
+      </c>
+      <c r="B100" t="n">
+        <v>50</v>
       </c>
       <c r="C100"/>
       <c r="D100"/>
       <c r="E100" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>83</v>
+        <v>85</v>
+      </c>
+      <c r="B101" t="n">
+        <v>1047</v>
       </c>
       <c r="C101"/>
       <c r="D101"/>
       <c r="E101" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="s">
-        <v>84</v>
-      </c>
-      <c r="C102"/>
-      <c r="D102"/>
-      <c r="E102" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="103">
-      <c r="A103" t="s">
-        <v>85</v>
-      </c>
-      <c r="C103"/>
-      <c r="D103"/>
-      <c r="E103" t="s">
-        <v>78</v>
+      <c r="A103" s="2" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>86</v>
+        <v>87</v>
+      </c>
+      <c r="B104" t="n">
+        <v>108</v>
       </c>
       <c r="C104"/>
       <c r="D104"/>
       <c r="E104" t="s">
-        <v>78</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="s">
+        <v>89</v>
+      </c>
+      <c r="B105" t="n">
+        <v>1032</v>
+      </c>
+      <c r="C105"/>
+      <c r="D105"/>
+      <c r="E105" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="s">
-        <v>87</v>
+      <c r="A106" t="s">
+        <v>91</v>
+      </c>
+      <c r="B106"/>
+      <c r="C106"/>
+      <c r="D106"/>
+      <c r="E106" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B107" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="C107"/>
       <c r="D107"/>
       <c r="E107" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B108" t="n">
-        <v>1032</v>
+        <v>15</v>
       </c>
       <c r="C108"/>
       <c r="D108"/>
       <c r="E108" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>92</v>
+        <v>94</v>
+      </c>
+      <c r="B109" t="n">
+        <v>1</v>
       </c>
       <c r="C109"/>
       <c r="D109"/>
       <c r="E109" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B110" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="C110"/>
       <c r="D110"/>
       <c r="E110" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B111" t="n">
-        <v>15</v>
+        <v>-106</v>
       </c>
       <c r="C111"/>
       <c r="D111"/>
       <c r="E111" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B112" t="n">
-        <v>1</v>
+        <v>-54</v>
       </c>
       <c r="C112"/>
       <c r="D112"/>
       <c r="E112" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B113" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="C113"/>
       <c r="D113"/>
       <c r="E113" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B114" t="n">
-        <v>-106</v>
+        <v>-76</v>
       </c>
       <c r="C114"/>
       <c r="D114"/>
       <c r="E114" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B115" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C115"/>
       <c r="D115"/>
       <c r="E115" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B116" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C116"/>
       <c r="D116"/>
       <c r="E116" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B117" t="n">
-        <v>-76</v>
+        <v>3</v>
       </c>
       <c r="C117"/>
       <c r="D117"/>
       <c r="E117" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>101</v>
+        <v>103</v>
+      </c>
+      <c r="B118" t="n">
+        <v>1044</v>
       </c>
       <c r="C118"/>
       <c r="D118"/>
       <c r="E118" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="s">
-        <v>102</v>
-      </c>
-      <c r="C119"/>
-      <c r="D119"/>
-      <c r="E119" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="s">
-        <v>103</v>
-      </c>
-      <c r="B120" t="n">
-        <v>-5</v>
-      </c>
-      <c r="C120"/>
-      <c r="D120"/>
-      <c r="E120" t="s">
-        <v>91</v>
+      <c r="A120" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>104</v>
-      </c>
-      <c r="B121" t="n">
-        <v>3</v>
+        <v>105</v>
       </c>
       <c r="C121"/>
       <c r="D121"/>
       <c r="E121" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>105</v>
-      </c>
-      <c r="B122" t="n">
-        <v>1044</v>
+        <v>107</v>
       </c>
       <c r="C122"/>
       <c r="D122"/>
       <c r="E122" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="s">
         <v>106</v>
-      </c>
-      <c r="C123"/>
-      <c r="D123"/>
-      <c r="E123" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>108</v>
+        <v>78</v>
       </c>
       <c r="C126"/>
       <c r="D126"/>
       <c r="E126" t="s">
-        <v>109</v>
+        <v>79</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>110</v>
+        <v>80</v>
       </c>
       <c r="C127"/>
       <c r="D127"/>
       <c r="E127" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="s">
         <v>109</v>
       </c>
+      <c r="B128" t="n">
+        <v>45</v>
+      </c>
+      <c r="C128"/>
+      <c r="D128"/>
+      <c r="E128" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="s">
+        <v>110</v>
+      </c>
+      <c r="C129"/>
+      <c r="D129"/>
+      <c r="E129" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="s">
+      <c r="A130" t="s">
         <v>111</v>
+      </c>
+      <c r="C130"/>
+      <c r="D130"/>
+      <c r="E130" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>77</v>
+        <v>112</v>
       </c>
       <c r="C131"/>
       <c r="D131"/>
       <c r="E131" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="C132"/>
       <c r="D132"/>
       <c r="E132" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="C133"/>
       <c r="D133"/>
       <c r="E133" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>112</v>
+        <v>115</v>
+      </c>
+      <c r="B134" t="n">
+        <v>-7</v>
       </c>
       <c r="C134"/>
       <c r="D134"/>
       <c r="E134" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C135"/>
       <c r="D135"/>
       <c r="E135" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C136"/>
       <c r="D136"/>
       <c r="E136" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="s">
-        <v>115</v>
-      </c>
-      <c r="C137"/>
-      <c r="D137"/>
-      <c r="E137" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>116</v>
+        <v>118</v>
+      </c>
+      <c r="B138" t="s">
+        <v>119</v>
       </c>
       <c r="C138"/>
       <c r="D138"/>
-      <c r="E138" t="s">
-        <v>78</v>
-      </c>
     </row>
     <row r="139">
-      <c r="A139" t="s">
-        <v>117</v>
-      </c>
-      <c r="C139"/>
-      <c r="D139"/>
-      <c r="E139" t="s">
-        <v>78</v>
+      <c r="A139" s="2" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>118</v>
+        <v>121</v>
+      </c>
+      <c r="B140" t="n">
+        <v>81</v>
       </c>
       <c r="C140"/>
       <c r="D140"/>
       <c r="E140" t="s">
-        <v>78</v>
+        <v>122</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>119</v>
+        <v>123</v>
+      </c>
+      <c r="B141" t="n">
+        <v>697</v>
       </c>
       <c r="C141"/>
       <c r="D141"/>
       <c r="E141" t="s">
-        <v>78</v>
+        <v>124</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="s">
+        <v>92</v>
+      </c>
+      <c r="B142" t="n">
+        <v>6</v>
+      </c>
+      <c r="C142"/>
+      <c r="D142"/>
+      <c r="E142" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>120</v>
-      </c>
-      <c r="B143" t="s">
-        <v>121</v>
+        <v>93</v>
+      </c>
+      <c r="B143" t="n">
+        <v>56</v>
       </c>
       <c r="C143"/>
       <c r="D143"/>
+      <c r="E143" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="s">
+      <c r="A144" t="s">
+        <v>94</v>
+      </c>
+      <c r="C144"/>
+      <c r="D144"/>
+      <c r="E144" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>123</v>
+        <v>95</v>
       </c>
       <c r="B145" t="n">
-        <v>122</v>
+        <v>-113</v>
       </c>
       <c r="C145"/>
       <c r="D145"/>
@@ -2271,17 +2362,20 @@
         <v>125</v>
       </c>
       <c r="B146" t="n">
-        <v>697</v>
+        <v>-6</v>
       </c>
       <c r="C146"/>
       <c r="D146"/>
       <c r="E146" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>93</v>
+        <v>126</v>
+      </c>
+      <c r="B147" t="n">
+        <v>-72</v>
       </c>
       <c r="C147"/>
       <c r="D147"/>
@@ -2291,23 +2385,23 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="B148" t="n">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="C148"/>
       <c r="D148"/>
       <c r="E148" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>95</v>
+        <v>128</v>
       </c>
       <c r="B149" t="n">
-        <v>5</v>
+        <v>584</v>
       </c>
       <c r="C149"/>
       <c r="D149"/>
@@ -2315,276 +2409,252 @@
         <v>124</v>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" t="s">
-        <v>96</v>
-      </c>
-      <c r="B150" t="n">
-        <v>-113</v>
-      </c>
-      <c r="C150"/>
-      <c r="D150"/>
-      <c r="E150" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="s">
-        <v>127</v>
-      </c>
-      <c r="B151" t="n">
-        <v>-3</v>
-      </c>
-      <c r="C151"/>
-      <c r="D151"/>
-      <c r="E151" t="s">
-        <v>124</v>
-      </c>
-    </row>
     <row r="152">
-      <c r="A152" t="s">
-        <v>128</v>
-      </c>
-      <c r="B152" t="n">
-        <v>-72</v>
-      </c>
-      <c r="C152"/>
-      <c r="D152"/>
-      <c r="E152" t="s">
-        <v>126</v>
+      <c r="A152" s="2" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>129</v>
-      </c>
-      <c r="B153" t="n">
-        <v>117</v>
+        <v>78</v>
       </c>
       <c r="C153"/>
       <c r="D153"/>
       <c r="E153" t="s">
-        <v>124</v>
+        <v>79</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="s">
         <v>130</v>
       </c>
-      <c r="B154" t="n">
-        <v>584</v>
-      </c>
       <c r="C154"/>
       <c r="D154"/>
       <c r="E154" t="s">
-        <v>126</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="s">
+        <v>131</v>
+      </c>
+      <c r="C155"/>
+      <c r="D155"/>
+      <c r="E155" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="s">
+        <v>132</v>
+      </c>
+      <c r="C156"/>
+      <c r="D156"/>
+      <c r="E156" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="s">
-        <v>131</v>
+      <c r="A157" t="s">
+        <v>133</v>
+      </c>
+      <c r="C157"/>
+      <c r="D157"/>
+      <c r="E157" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>77</v>
+        <v>110</v>
       </c>
       <c r="C158"/>
       <c r="D158"/>
       <c r="E158" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C159"/>
       <c r="D159"/>
       <c r="E159" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C160"/>
       <c r="D160"/>
       <c r="E160" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="s">
-        <v>134</v>
-      </c>
-      <c r="C161"/>
-      <c r="D161"/>
-      <c r="E161" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="162">
-      <c r="A162" t="s">
-        <v>135</v>
-      </c>
-      <c r="C162"/>
-      <c r="D162"/>
-      <c r="E162" t="s">
-        <v>78</v>
+      <c r="A162" s="2" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>112</v>
+        <v>78</v>
       </c>
       <c r="C163"/>
       <c r="D163"/>
       <c r="E163" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C164"/>
       <c r="D164"/>
       <c r="E164" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C165"/>
       <c r="D165"/>
       <c r="E165" t="s">
-        <v>78</v>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="s">
+        <v>137</v>
+      </c>
+      <c r="C166"/>
+      <c r="D166"/>
+      <c r="E166" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="s">
+      <c r="A167" t="s">
+        <v>135</v>
+      </c>
+      <c r="C167"/>
+      <c r="D167"/>
+      <c r="E167" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="s">
         <v>138</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="s">
-        <v>77</v>
-      </c>
-      <c r="C168"/>
-      <c r="D168"/>
-      <c r="E168" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="s">
-        <v>132</v>
-      </c>
-      <c r="C169"/>
-      <c r="D169"/>
-      <c r="E169" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>135</v>
+        <v>139</v>
+      </c>
+      <c r="B170" t="n">
+        <v>97</v>
       </c>
       <c r="C170"/>
       <c r="D170"/>
       <c r="E170" t="s">
-        <v>78</v>
+        <v>140</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>139</v>
+        <v>141</v>
+      </c>
+      <c r="B171" t="n">
+        <v>203</v>
       </c>
       <c r="C171"/>
       <c r="D171"/>
       <c r="E171" t="s">
-        <v>78</v>
+        <v>140</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C172"/>
       <c r="D172"/>
       <c r="E172" t="s">
-        <v>78</v>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="s">
+        <v>143</v>
+      </c>
+      <c r="B173" t="n">
+        <v>-8</v>
+      </c>
+      <c r="C173"/>
+      <c r="D173"/>
+      <c r="E173" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="s">
+      <c r="A174" t="s">
+        <v>144</v>
+      </c>
+      <c r="B174" t="n">
+        <v>195</v>
+      </c>
+      <c r="C174"/>
+      <c r="D174"/>
+      <c r="E174" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B175" t="n">
-        <v>97</v>
+        <v>4</v>
       </c>
       <c r="C175"/>
       <c r="D175"/>
       <c r="E175" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>143</v>
-      </c>
-      <c r="B176" t="n">
-        <v>203</v>
+        <v>134</v>
       </c>
       <c r="C176"/>
       <c r="D176"/>
       <c r="E176" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>144</v>
+        <v>145</v>
+      </c>
+      <c r="B177" t="n">
+        <v>296</v>
       </c>
       <c r="C177"/>
       <c r="D177"/>
       <c r="E177" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="s">
-        <v>145</v>
-      </c>
-      <c r="B178" t="n">
-        <v>-8</v>
-      </c>
-      <c r="C178"/>
-      <c r="D178"/>
-      <c r="E178" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="s">
+      <c r="A179" s="2" t="s">
         <v>146</v>
-      </c>
-      <c r="B179" t="n">
-        <v>203</v>
-      </c>
-      <c r="C179"/>
-      <c r="D179"/>
-      <c r="E179" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="180">
@@ -2592,602 +2662,641 @@
         <v>139</v>
       </c>
       <c r="B180" t="n">
-        <v>4</v>
+        <v>79</v>
       </c>
       <c r="C180"/>
       <c r="D180"/>
       <c r="E180" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>136</v>
+        <v>147</v>
+      </c>
+      <c r="B181" t="n">
+        <v>17</v>
       </c>
       <c r="C181"/>
       <c r="D181"/>
       <c r="E181" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="B182" t="n">
-        <v>296</v>
+        <v>-2</v>
       </c>
       <c r="C182"/>
       <c r="D182"/>
       <c r="E182" t="s">
-        <v>142</v>
+        <v>122</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="s">
+        <v>134</v>
+      </c>
+      <c r="B183" t="n">
+        <v>-8</v>
+      </c>
+      <c r="C183"/>
+      <c r="D183"/>
+      <c r="E183" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="s">
+      <c r="A184" t="s">
+        <v>145</v>
+      </c>
+      <c r="B184" t="n">
+        <v>86</v>
+      </c>
+      <c r="C184"/>
+      <c r="D184"/>
+      <c r="E184" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="s">
         <v>148</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="s">
-        <v>141</v>
-      </c>
-      <c r="C185"/>
-      <c r="D185"/>
-      <c r="E185" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="s">
-        <v>149</v>
-      </c>
-      <c r="C186"/>
-      <c r="D186"/>
-      <c r="E186" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="s">
         <v>139</v>
       </c>
+      <c r="B187" t="n">
+        <v>142</v>
+      </c>
       <c r="C187"/>
       <c r="D187"/>
       <c r="E187" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>136</v>
+        <v>141</v>
+      </c>
+      <c r="B188" t="n">
+        <v>-77</v>
       </c>
       <c r="C188"/>
       <c r="D188"/>
       <c r="E188" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>147</v>
+        <v>144</v>
+      </c>
+      <c r="B189" t="n">
+        <v>-77</v>
       </c>
       <c r="C189"/>
       <c r="D189"/>
       <c r="E189" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="s">
+        <v>145</v>
+      </c>
+      <c r="B190" t="n">
+        <v>65</v>
+      </c>
+      <c r="C190"/>
+      <c r="D190"/>
+      <c r="E190" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" t="s">
-        <v>141</v>
-      </c>
-      <c r="B192" t="n">
-        <v>142</v>
-      </c>
-      <c r="C192"/>
-      <c r="D192"/>
-      <c r="E192" t="s">
+    <row r="195">
+      <c r="A195" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" t="s">
-        <v>143</v>
-      </c>
-      <c r="B193" t="n">
-        <v>-77</v>
-      </c>
-      <c r="C193"/>
-      <c r="D193"/>
-      <c r="E193" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="s">
-        <v>146</v>
-      </c>
-      <c r="B194" t="n">
-        <v>-77</v>
-      </c>
-      <c r="C194"/>
-      <c r="D194"/>
-      <c r="E194" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="s">
-        <v>147</v>
-      </c>
-      <c r="B195" t="n">
-        <v>65</v>
-      </c>
-      <c r="C195"/>
-      <c r="D195"/>
-      <c r="E195" t="s">
-        <v>151</v>
+    <row r="196">
+      <c r="A196" t="s">
+        <v>152</v>
+      </c>
+      <c r="B196" t="n">
+        <v>1.93</v>
+      </c>
+      <c r="C196"/>
+      <c r="D196"/>
+      <c r="E196" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="s">
+        <v>154</v>
+      </c>
+      <c r="C197"/>
+      <c r="D197"/>
+      <c r="E197" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="s">
-        <v>152</v>
+      <c r="A198" t="s">
+        <v>155</v>
+      </c>
+      <c r="B198" t="n">
+        <v>5709</v>
+      </c>
+      <c r="C198"/>
+      <c r="D198"/>
+      <c r="E198" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="s">
+        <v>156</v>
+      </c>
+      <c r="B199" t="n">
+        <v>11013</v>
+      </c>
+      <c r="C199"/>
+      <c r="D199"/>
+      <c r="E199" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="s">
-        <v>153</v>
+      <c r="A200" t="s">
+        <v>157</v>
+      </c>
+      <c r="B200"/>
+      <c r="C200"/>
+      <c r="D200"/>
+      <c r="E200" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B201" t="n">
-        <v>1.93</v>
+        <v>5304</v>
       </c>
       <c r="C201"/>
       <c r="D201"/>
       <c r="E201" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>156</v>
+        <v>160</v>
+      </c>
+      <c r="B202" t="n">
+        <v>504</v>
       </c>
       <c r="C202"/>
       <c r="D202"/>
       <c r="E202" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="s">
-        <v>157</v>
-      </c>
-      <c r="B203" t="n">
-        <v>5709</v>
-      </c>
-      <c r="C203"/>
-      <c r="D203"/>
-      <c r="E203" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="s">
-        <v>158</v>
-      </c>
-      <c r="B204" t="n">
-        <v>11013</v>
-      </c>
-      <c r="C204"/>
-      <c r="D204"/>
-      <c r="E204" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="s">
-        <v>159</v>
-      </c>
-      <c r="B205"/>
-      <c r="C205"/>
-      <c r="D205"/>
-      <c r="E205" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="s">
+      <c r="A205" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B206" t="n">
-        <v>5304</v>
-      </c>
-      <c r="C206"/>
-      <c r="D206"/>
-      <c r="E206" t="s">
-        <v>160</v>
-      </c>
     </row>
     <row r="207">
-      <c r="A207" t="s">
+      <c r="A207" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B207" t="n">
-        <v>504</v>
-      </c>
-      <c r="C207"/>
-      <c r="D207"/>
-      <c r="E207" t="s">
-        <v>155</v>
+    </row>
+    <row r="208">
+      <c r="A208" t="s">
+        <v>163</v>
+      </c>
+      <c r="B208" t="n">
+        <v>10596</v>
+      </c>
+      <c r="C208"/>
+      <c r="D208"/>
+      <c r="E208" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="s">
+        <v>165</v>
+      </c>
+      <c r="B209" t="n">
+        <v>10837</v>
+      </c>
+      <c r="C209"/>
+      <c r="D209"/>
+      <c r="E209" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="s">
-        <v>163</v>
+      <c r="A210" t="s">
+        <v>166</v>
+      </c>
+      <c r="B210" t="n">
+        <v>2582</v>
+      </c>
+      <c r="C210"/>
+      <c r="D210"/>
+      <c r="E210" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="s">
+        <v>167</v>
+      </c>
+      <c r="B211" t="n">
+        <v>14205</v>
+      </c>
+      <c r="C211"/>
+      <c r="D211"/>
+      <c r="E211" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="s">
+      <c r="A212" t="s">
+        <v>168</v>
+      </c>
+      <c r="B212" t="n">
+        <v>467</v>
+      </c>
+      <c r="C212"/>
+      <c r="D212"/>
+      <c r="E212" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B213" t="n">
-        <v>10596</v>
+        <v>8207</v>
       </c>
       <c r="C213"/>
       <c r="D213"/>
       <c r="E213" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B214" t="n">
-        <v>10837</v>
+        <v>262</v>
       </c>
       <c r="C214"/>
       <c r="D214"/>
       <c r="E214" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B215" t="n">
-        <v>2582</v>
+        <v>1656</v>
       </c>
       <c r="C215"/>
       <c r="D215"/>
       <c r="E215" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B216" t="n">
-        <v>14205</v>
+        <v>38216</v>
       </c>
       <c r="C216"/>
       <c r="D216"/>
       <c r="E216" t="s">
-        <v>166</v>
+        <v>14</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B217" t="n">
-        <v>467</v>
+        <v>4498</v>
       </c>
       <c r="C217"/>
       <c r="D217"/>
       <c r="E217" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B218" t="n">
-        <v>8207</v>
+        <v>4885</v>
       </c>
       <c r="C218"/>
       <c r="D218"/>
       <c r="E218" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B219" t="n">
-        <v>262</v>
+        <v>58195</v>
       </c>
       <c r="C219"/>
       <c r="D219"/>
       <c r="E219" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="s">
-        <v>173</v>
-      </c>
-      <c r="B220" t="n">
-        <v>1656</v>
-      </c>
-      <c r="C220"/>
-      <c r="D220"/>
-      <c r="E220" t="s">
-        <v>166</v>
+        <v>14</v>
       </c>
     </row>
     <row r="221">
-      <c r="A221" t="s">
-        <v>174</v>
-      </c>
-      <c r="B221" t="n">
-        <v>38216</v>
-      </c>
-      <c r="C221"/>
-      <c r="D221"/>
-      <c r="E221" t="s">
-        <v>14</v>
+      <c r="A221" s="2" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B222" t="n">
-        <v>4498</v>
+        <v>18556</v>
       </c>
       <c r="C222"/>
       <c r="D222"/>
       <c r="E222" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B223" t="n">
-        <v>4885</v>
+        <v>372</v>
       </c>
       <c r="C223"/>
       <c r="D223"/>
       <c r="E223" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>177</v>
-      </c>
-      <c r="B224" t="n">
-        <v>58195</v>
+        <v>179</v>
       </c>
       <c r="C224"/>
       <c r="D224"/>
       <c r="E224" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="s">
+        <v>180</v>
+      </c>
+      <c r="B225" t="n">
+        <v>18928</v>
+      </c>
+      <c r="C225"/>
+      <c r="D225"/>
+      <c r="E225" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="s">
-        <v>178</v>
+      <c r="A226" t="s">
+        <v>181</v>
+      </c>
+      <c r="B226" t="n">
+        <v>294</v>
+      </c>
+      <c r="C226"/>
+      <c r="D226"/>
+      <c r="E226" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B227" t="n">
-        <v>18556</v>
+        <v>84</v>
       </c>
       <c r="C227"/>
       <c r="D227"/>
       <c r="E227" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B228" t="n">
-        <v>372</v>
+        <v>19306</v>
       </c>
       <c r="C228"/>
       <c r="D228"/>
       <c r="E228" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="s">
-        <v>181</v>
-      </c>
-      <c r="C229"/>
-      <c r="D229"/>
-      <c r="E229" t="s">
-        <v>166</v>
+        <v>14</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>182</v>
-      </c>
-      <c r="B230" t="n">
-        <v>18928</v>
+        <v>184</v>
       </c>
       <c r="C230"/>
       <c r="D230"/>
       <c r="E230" t="s">
-        <v>14</v>
+        <v>185</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B231" t="n">
-        <v>294</v>
+        <v>77501</v>
       </c>
       <c r="C231"/>
       <c r="D231"/>
       <c r="E231" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="s">
-        <v>184</v>
-      </c>
-      <c r="B232" t="n">
-        <v>84</v>
-      </c>
-      <c r="C232"/>
-      <c r="D232"/>
-      <c r="E232" t="s">
-        <v>166</v>
+        <v>14</v>
       </c>
     </row>
     <row r="233">
-      <c r="A233" t="s">
-        <v>185</v>
-      </c>
-      <c r="B233" t="n">
-        <v>19306</v>
-      </c>
-      <c r="C233"/>
-      <c r="D233"/>
-      <c r="E233" t="s">
-        <v>14</v>
+      <c r="A233" s="2" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="s">
+        <v>188</v>
+      </c>
+      <c r="C234"/>
+      <c r="D234"/>
+      <c r="E234" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>186</v>
+        <v>189</v>
+      </c>
+      <c r="B235" t="n">
+        <v>59217</v>
       </c>
       <c r="C235"/>
       <c r="D235"/>
       <c r="E235" t="s">
-        <v>187</v>
+        <v>164</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B236" t="n">
-        <v>77501</v>
+        <v>18284</v>
       </c>
       <c r="C236"/>
       <c r="D236"/>
       <c r="E236" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" s="2" t="s">
-        <v>189</v>
+        <v>164</v>
       </c>
     </row>
     <row r="239">
-      <c r="A239" t="s">
-        <v>190</v>
-      </c>
-      <c r="C239"/>
-      <c r="D239"/>
-      <c r="E239" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="s">
+      <c r="A239" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B240" t="n">
-        <v>59217</v>
-      </c>
-      <c r="C240"/>
-      <c r="D240"/>
-      <c r="E240" t="s">
-        <v>166</v>
-      </c>
     </row>
     <row r="241">
-      <c r="A241" t="s">
+      <c r="A241" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="B241" t="n">
-        <v>18284</v>
-      </c>
-      <c r="C241"/>
-      <c r="D241"/>
-      <c r="E241" t="s">
-        <v>166</v>
+    </row>
+    <row r="242">
+      <c r="A242" t="s">
+        <v>193</v>
+      </c>
+      <c r="B242" t="n">
+        <v>2842</v>
+      </c>
+      <c r="C242"/>
+      <c r="D242"/>
+      <c r="E242" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="s">
+        <v>167</v>
+      </c>
+      <c r="B243" t="n">
+        <v>16852</v>
+      </c>
+      <c r="C243"/>
+      <c r="D243"/>
+      <c r="E243" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="s">
-        <v>193</v>
+      <c r="A244" t="s">
+        <v>195</v>
+      </c>
+      <c r="B244" t="n">
+        <v>8522</v>
+      </c>
+      <c r="C244"/>
+      <c r="D244"/>
+      <c r="E244" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="s">
+        <v>169</v>
+      </c>
+      <c r="B245" t="n">
+        <v>8207</v>
+      </c>
+      <c r="C245"/>
+      <c r="D245"/>
+      <c r="E245" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="246">
-      <c r="A246" s="2" t="s">
+      <c r="A246" t="s">
+        <v>177</v>
+      </c>
+      <c r="B246" t="n">
+        <v>18556</v>
+      </c>
+      <c r="C246"/>
+      <c r="D246"/>
+      <c r="E246" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="B247" t="n">
-        <v>2842</v>
+        <v>1713</v>
       </c>
       <c r="C247"/>
       <c r="D247"/>
       <c r="E247" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>169</v>
+        <v>196</v>
       </c>
       <c r="B248" t="n">
-        <v>16852</v>
+        <v>663</v>
       </c>
       <c r="C248"/>
       <c r="D248"/>
       <c r="E248" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="249">
@@ -3195,246 +3304,181 @@
         <v>197</v>
       </c>
       <c r="B249" t="n">
-        <v>8522</v>
+        <v>3520</v>
       </c>
       <c r="C249"/>
       <c r="D249"/>
       <c r="E249" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>171</v>
+        <v>198</v>
       </c>
       <c r="B250" t="n">
-        <v>8207</v>
+        <v>71057</v>
       </c>
       <c r="C250"/>
       <c r="D250"/>
       <c r="E250" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="s">
-        <v>179</v>
-      </c>
-      <c r="B251" t="n">
-        <v>18556</v>
-      </c>
-      <c r="C251"/>
-      <c r="D251"/>
-      <c r="E251" t="s">
-        <v>196</v>
+        <v>14</v>
       </c>
     </row>
     <row r="252">
-      <c r="A252" t="s">
-        <v>186</v>
-      </c>
-      <c r="B252" t="n">
-        <v>1713</v>
-      </c>
-      <c r="C252"/>
-      <c r="D252"/>
-      <c r="E252" t="s">
-        <v>196</v>
+      <c r="A252" s="2" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B253" t="n">
-        <v>663</v>
+        <v>3636</v>
       </c>
       <c r="C253"/>
       <c r="D253"/>
       <c r="E253" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>199</v>
+        <v>167</v>
       </c>
       <c r="B254" t="n">
-        <v>3520</v>
+        <v>537</v>
       </c>
       <c r="C254"/>
       <c r="D254"/>
       <c r="E254" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B255" t="n">
-        <v>71057</v>
+        <v>1758</v>
       </c>
       <c r="C255"/>
       <c r="D255"/>
       <c r="E255" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="s">
+        <v>197</v>
+      </c>
+      <c r="B256" t="n">
+        <v>524</v>
+      </c>
+      <c r="C256"/>
+      <c r="D256"/>
+      <c r="E256" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="s">
+        <v>202</v>
+      </c>
+      <c r="B257" t="n">
+        <v>7234</v>
+      </c>
+      <c r="C257"/>
+      <c r="D257"/>
+      <c r="E257" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="257">
-      <c r="A257" s="2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="s">
-        <v>202</v>
-      </c>
-      <c r="B258" t="n">
-        <v>3636</v>
-      </c>
-      <c r="C258"/>
-      <c r="D258"/>
-      <c r="E258" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="s">
-        <v>169</v>
-      </c>
-      <c r="B259" t="n">
-        <v>537</v>
-      </c>
-      <c r="C259"/>
-      <c r="D259"/>
-      <c r="E259" t="s">
-        <v>196</v>
-      </c>
-    </row>
     <row r="260">
-      <c r="A260" t="s">
+      <c r="A260" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="B260" t="n">
-        <v>1758</v>
-      </c>
-      <c r="C260"/>
-      <c r="D260"/>
-      <c r="E260" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>199</v>
-      </c>
-      <c r="B261" t="n">
-        <v>524</v>
+        <v>204</v>
       </c>
       <c r="C261"/>
       <c r="D261"/>
       <c r="E261" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B262" t="n">
-        <v>7234</v>
+        <v>2170</v>
       </c>
       <c r="C262"/>
       <c r="D262"/>
       <c r="E262" t="s">
-        <v>14</v>
+        <v>205</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="s">
+        <v>207</v>
+      </c>
+      <c r="B263" t="n">
+        <v>18542</v>
+      </c>
+      <c r="C263"/>
+      <c r="D263"/>
+      <c r="E263" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="s">
+        <v>208</v>
+      </c>
+      <c r="B264" t="n">
+        <v>4593</v>
+      </c>
+      <c r="C264"/>
+      <c r="D264"/>
+      <c r="E264" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="265">
-      <c r="A265" s="2" t="s">
+      <c r="A265" t="s">
+        <v>209</v>
+      </c>
+      <c r="C265"/>
+      <c r="D265"/>
+      <c r="E265" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C266"/>
       <c r="D266"/>
       <c r="E266" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B267" t="n">
-        <v>2170</v>
+        <v>27526</v>
       </c>
       <c r="C267"/>
       <c r="D267"/>
       <c r="E267" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="s">
-        <v>209</v>
-      </c>
-      <c r="B268" t="n">
-        <v>18542</v>
-      </c>
-      <c r="C268"/>
-      <c r="D268"/>
-      <c r="E268" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="s">
-        <v>210</v>
-      </c>
-      <c r="B269" t="n">
-        <v>4593</v>
-      </c>
-      <c r="C269"/>
-      <c r="D269"/>
-      <c r="E269" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="s">
-        <v>211</v>
-      </c>
-      <c r="C270"/>
-      <c r="D270"/>
-      <c r="E270" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="s">
-        <v>212</v>
-      </c>
-      <c r="C271"/>
-      <c r="D271"/>
-      <c r="E271" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="s">
-        <v>213</v>
-      </c>
-      <c r="B272" t="n">
-        <v>27526</v>
-      </c>
-      <c r="C272"/>
-      <c r="D272"/>
-      <c r="E272" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>